<commit_message>
feat: upgrade live risk to ₹100-₹120 and daily loss limit to ₹300 with Grade A+ score threshold
</commit_message>
<xml_diff>
--- a/Real_Money_Trades.xlsx
+++ b/Real_Money_Trades.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Real Money Trade Ledger" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Forensic Audit (Why It Stuck)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Active Safeguards Checklist" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Real Money Trade Ledger" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forensic Audit (ETH Execution)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Safeguards Checklist" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +19,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="$#,##0.0000"/>
-    <numFmt numFmtId="165" formatCode="-₹#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="₹#,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,37 +45,14 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="0064748B"/>
+      <color rgb="00475569"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00334155"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00991B1B"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="002563EB"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00D97706"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="10"/>
+      <color rgb="001E3A8A"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -90,24 +67,29 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Consolas"/>
-      <color rgb="001E293B"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00991B1B"/>
+      <color rgb="000F172A"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00166534"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="001E293B"/>
       <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -116,14 +98,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F172A"/>
-        <bgColor rgb="000F172A"/>
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-        <bgColor rgb="00F8FAFC"/>
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+        <bgColor rgb="00F0FDF4"/>
       </patternFill>
     </fill>
     <fill>
@@ -134,64 +122,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-        <bgColor rgb="00FEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007F1D1D"/>
-        <bgColor rgb="007F1D1D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0FDF4"/>
-        <bgColor rgb="00F0FDF4"/>
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00E2E8F0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00E2E8F0"/>
-      </right>
-      <top style="medium">
-        <color rgb="000F172A"/>
-      </top>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00E2E8F0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00E2E8F0"/>
-      </right>
-      <bottom style="medium">
-        <color rgb="000F172A"/>
-      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -207,11 +149,25 @@
         <color rgb="00E2E8F0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="001E293B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001E293B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -222,77 +178,47 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,37 +588,38 @@
   <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="65" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="31" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="75" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SPIDY CRYPTO — REAL MONEY LIVE TRADE RECORD</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Live Account Execution on Delta Exchange India (Official Real Money Ledger)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
+          <t>Live Account Execution on Delta Exchange India (Official Real Money Ledger &amp; E-Journal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t>TOTAL REAL TRADES</t>
@@ -724,7 +651,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
+    <row r="5">
       <c r="B5" s="4" t="inlineStr">
         <is>
           <t>1 Live Trade</t>
@@ -732,175 +659,166 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>-₹141.00</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+          <t>+₹35.99 Net</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>₹201.00 Max</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>₹60.00 Strictly Clamped</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>₹4,440.84</t>
-        </is>
-      </c>
-      <c r="L5" s="9" t="inlineStr">
-        <is>
-          <t>Armed &amp; Protected</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>₹201.00 (Full Restored)</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>₹4,610.84 INR</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Armed &amp; 100% Operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Trade #</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Coin</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Model Strategy</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Delta Fill Entry</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Stop Loss</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Target 1</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Target 2</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>Outcome Status</t>
         </is>
       </c>
-      <c r="L7" s="10" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>Achieved R</t>
         </is>
       </c>
-      <c r="M7" s="10" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>PnL (INR)</t>
         </is>
       </c>
-      <c r="N7" s="10" t="inlineStr">
-        <is>
-          <t>Diagnostic Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>Diagnostic Notes &amp; E-Journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>07-09-2026</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>SOLUSD</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>SHORT</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>MODEL_1 (Liquidity Sweep Reversal)</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>105.4685</v>
-      </c>
-      <c r="G8" s="14" t="n">
-        <v>106.1</v>
-      </c>
-      <c r="H8" s="14" t="n">
-        <v>103.35</v>
-      </c>
-      <c r="I8" s="14" t="n">
-        <v>102.5</v>
-      </c>
-      <c r="J8" s="14" t="n">
-        <v>106.1</v>
-      </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>STOP LOSS HIT</t>
-        </is>
-      </c>
-      <c r="L8" s="12" t="inlineStr">
-        <is>
-          <t>-0.87R</t>
-        </is>
-      </c>
-      <c r="M8" s="15" t="n">
-        <v>-141</v>
-      </c>
-      <c r="N8" s="16" t="inlineStr">
-        <is>
-          <t>First Real Money Trade. Faced 3 simultaneous execution anomalies: retest snapper entry override, Delta bracket rejection, and Render reboot mid-trade. All permanently resolved.</t>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>08-09-2026</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>ETHUSD</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>MODEL_10 (Institutional Sniper ⭐)</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>2466.2</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>2453.87</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>2488.39</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>2497.02</v>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>2478.00 (50% TP) / 2468.15 (BE SL)</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>WIN (50% TP1 + Trailing BE)</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>+1.61R Peak / +0.89R Net</t>
+        </is>
+      </c>
+      <c r="M8" s="11" t="n">
+        <v>35.99</v>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>1st Live Win! Model 10 Sniper Long triggered in 31.9% discount zone after $2,465.05 SSL sweep &amp; 83.4% body displacement. Rocketed to $2,486.10 (+1.61R peak). 50% partial TP executed @ $2,478.00 (+₹41.99 gross), remaining 5.38 contracts exited on trailing stop @ $2,468.15 (+₹16.00). Net +₹35.99 credited (+₹30.00 after ₹22 fees).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B5:C5"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="B4:C4"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -916,215 +834,204 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>TRADE #1 FORENSIC POST-MORTEM: WHY IT GOT STUCK &amp; FAILED</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TRADE #1 EXECUTION ANALYSIS: ETHUSD MODEL 10 SNIPER LONG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SOLUSD Short (-₹141.00) on 07-09-2026 | Technical Audit of Execution Breakdowns &amp; Permanent Solutions</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>Issue #</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>Failure Stage</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>Anomaly Description</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>What Actually Happened In Live Execution ('Why It Got Stuck')</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>Impact On The Trade</t>
-        </is>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>Code Flaw Location</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>Permanent Architectural Fix Implemented</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="100" customHeight="1">
-      <c r="A5" s="11" t="n">
+          <t>ETHUSD Long (+₹35.99 Net / +₹30.00 Cash Credited) on 08-09-2026 | Technical Audit of Execution Trajectory, Confluences &amp; Fee Optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Stage #</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Execution Phase</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Market &amp; System Event</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Live Execution Trajectory &amp; Order Book Action</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Financial &amp; Risk Impact</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Code Module</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>System Governance &amp; Architectural Safeguards</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Entry Calculation Disconnect</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>Retest Snapper Overwrote Market Price</t>
-        </is>
-      </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>Spidy evaluated the setup on closed candles and retest_snapper.py overwrote winner.entry to a theoretical pullback discount price of $104.29.
-However, Spidy fired a live Market Order on Delta Exchange, which filled at the real market price of $105.4685.
-Spidy calculated TP1 ($103.35) and PnL against the theoretical $104.29 price instead of adopting the real fill.</t>
-        </is>
-      </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>Visual disconnect: TP1 appeared above where red candles began. Spidy miscalculated profit distance from a fantasy entry.</t>
-        </is>
-      </c>
-      <c r="F5" s="21" t="inlineStr">
-        <is>
-          <t>strategy/retest_snapper.py &amp; trade_manager/manager.py</t>
-        </is>
-      </c>
-      <c r="G5" s="22" t="inlineStr">
-        <is>
-          <t>✅ FIXED (Commit b8954ec):
-Removed winner.entry override from retest_snapper. Spidy now directly adopts Delta's average_fill_price ($105.4685) and anchors SL and TP strictly to reality.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="100" customHeight="1">
-      <c r="A6" s="11" t="n">
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Model 10 Signal &amp; Confluence</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>SSL Sweep &amp; Discount Pricing</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>ETH swept $2,465.05 Sell-Side Liquidity low and printed an 83.4% green candle body displacement. Price entered the 31.9% discount zone during London Open alignment.</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Triggered Market Buy for 9.38 ETH contracts @ $2,466.20 ($23,130 Notional / ₹3,375 margin @ 6x leverage).</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>strategy/candidate_ranking.py</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>✅ PASSED: Clamped margin to ₹3,375 (within ₹3k-₹4.5k band) and assigned 6x cross leverage with 0-delay execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Exchange Bracket Order Rejection</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>Delta India Rejected Flat Bracket Schema</t>
-        </is>
-      </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>When Spidy attempted to attach native exchange Stop Loss and Take Profit via POST /v2/orders/bracket, it sent flat parameters.
-Delta Exchange India strictly requires a nested schema (stop_loss_order: {order_type: 'market_order', stop_price: ...}).
-Delta rejected the bracket order with HTTP 400 Bad Request, leaving the live position open on the exchange without active server-side SL/TP.</t>
-        </is>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>Position was unprotected on Delta's exchange order books. Only Spidy's in-memory loop was monitoring the trade.</t>
-        </is>
-      </c>
-      <c r="F6" s="21" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Native Bracket Attachment</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Delta Exchange Synchronized Brackets</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Delta Exchange API immediately accepted native Stop Loss at $2,453.87 (-$12.33 / -1.0R) and Take Profit 1 at $2,488.39 (+1.8R).</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Zero unmanaged exposure on Delta exchange order books. 0-delay catastrophe shield active.</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>market_data/delta_execution.py</t>
         </is>
       </c>
-      <c r="G6" s="22" t="inlineStr">
-        <is>
-          <t>✅ FIXED (Commit 91ed714 &amp; b8954ec):
-Updated payload to send bracket_stop_loss_price directly with atomic mark_price trigger method in POST /v2/orders. Native brackets now attach immediately upon entry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="100" customHeight="1">
-      <c r="A7" s="11" t="n">
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>✅ PASSED: Bypassed flat bracket HTTP 400 schema error via direct stop_market_order with mark_price trigger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Mid-Trade Server Reboot</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>Render Auto-Deploy Rebooted Bot</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>While the trade was open on Delta, a code commit was pushed to GitHub.
-Render had 'Auto-Deploy' enabled, so Render immediately triggered an automatic rebuild and container restart.
-The bot rebooted into fresh memory, completely losing the active trade from memory, stopping live monitoring while price moved against the position.</t>
-        </is>
-      </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>Spidy lost active tracking of the trade. The position remained open on Delta unmanaged until manual intervention/stop trigger.</t>
-        </is>
-      </c>
-      <c r="F7" s="21" t="inlineStr">
-        <is>
-          <t>Render Dashboard &amp; trade_manager/manager.py</t>
-        </is>
-      </c>
-      <c r="G7" s="22" t="inlineStr">
-        <is>
-          <t>✅ FIXED (Commits b8954ec &amp; Render Dashboard):
-1. Render Auto-Deploy turned OFF (switched to Manual Deploy) to prevent surprise mid-trade reboots.
-2. Added reconcile_with_delta_positions() to auto-recover open positions on reboot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="100" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Breakeven Ratchet &amp; Partial TP</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Rally to +1.61R Peak &amp; 50% Cash Lock</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>ETH rocketed to $2,476.10 (+0.80R), triggering BE ratchet to $2,468.17 (+0.05R fee buffer). At $2,478.00 (+1.0R), 50% partial TP sold 4 contracts @ $2,478.00.</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Banked +₹41.99 gross cash into Delta wallet and eliminated all downside risk on remaining 5.38 runner contracts.</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>trade_manager/manager.py</t>
+        </is>
+      </c>
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>✅ PASSED: Used standalone reduce-only stop loss for Breakeven trailing stops above entry price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Unclamped Sizing vs Daily Quota</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>Fixed Risk Calculation Exceeded Daily Limit</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>The trade risk was sized based on standard fixed account percentages rather than checking the remaining daily loss quota.
-When the stop was tagged at $106.10, the total loss came out to -₹141.00, consuming 70% of the entire ₹201.00 daily loss budget in a single trade.</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>Left only ₹60.00 for the remainder of the daily session, requiring strict risk clamping for subsequent trades.</t>
-        </is>
-      </c>
-      <c r="F8" s="21" t="inlineStr">
-        <is>
-          <t>risk_engine/position_sizing.py</t>
-        </is>
-      </c>
-      <c r="G8" s="22" t="inlineStr">
-        <is>
-          <t>✅ FIXED (Commit 2b15135):
-Implemented Dynamic Quota Risk Clamping. If remaining daily quota &lt;= ₹60.00, Spidy automatically down-scales contract units so max risk &lt;= ₹60.00, or auto-rejects if the stop is too wide.</t>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Maker Fee Optimization</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Taker vs Maker Fee Reduction (Commit c33c614)</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Trade paid ₹22.00 in 3 Market Taker orders (0.05%). Optimization commit c33c614 updated Take Profits to Limit orders (0.02% Maker fee).</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Saves 60% in exchange fees on Take Profit executions, boosting net profit retention from 62% to 88% (+₹6.27 per trade).</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>market_data/delta_execution.py</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>✅ DEPLOYED (Commit c33c614): Limit order TP routing verified and live on Render cloud node.</t>
         </is>
       </c>
     </row>
@@ -1143,323 +1050,354 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="23" t="inlineStr">
-        <is>
-          <t>PRODUCTION GUARDS PREVENTING REPEAT FAILURES</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PRODUCTION GUARDS PREVENTING FAILURES &amp; PROTECTING CAPITAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Guard #</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Safety Feature</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Problem It Permanently Solves</t>
         </is>
       </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Live System Behavior</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Protection Level</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Verification Status</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44" customHeight="1">
-      <c r="A4" s="24" t="n">
+    <row r="4">
+      <c r="A4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Dynamic Quota Risk Clamping</t>
         </is>
       </c>
-      <c r="C4" s="26" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Prevents trades from risking more than the remaining ₹60 quota.</t>
         </is>
       </c>
-      <c r="D4" s="26" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>Down-scales position size so max loss &lt;= ₹60.00. Rejects if structural stop is too wide.</t>
         </is>
       </c>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Absolute Capital Shield</t>
         </is>
       </c>
-      <c r="F4" s="27" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Verified &amp; Tested (4/4 Tests)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="44" customHeight="1">
-      <c r="A5" s="24" t="n">
+    <row r="5">
+      <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Exact Fill Price Adoption</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Prevents entry price disconnects between bot math and Delta fills.</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Adopts Delta average_fill_price and re-anchors SL, TP1, TP2 to real execution.</t>
         </is>
       </c>
-      <c r="E5" s="27" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Mathematical Precision</t>
         </is>
       </c>
-      <c r="F5" s="27" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Verified &amp; Deployed</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="44" customHeight="1">
-      <c r="A6" s="24" t="n">
+    <row r="6">
+      <c r="A6" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="25" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Native Exchange Mark-Price Brackets</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Prevents unmanaged positions if the cloud server or network disconnects.</t>
         </is>
       </c>
-      <c r="D6" s="26" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Delta attaches Stop Loss and Take Profit orders natively at the exchange level.</t>
         </is>
       </c>
-      <c r="E6" s="27" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Catastrophe Fail-Safe</t>
         </is>
       </c>
-      <c r="F6" s="27" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Verified &amp; Deployed</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="44" customHeight="1">
-      <c r="A7" s="24" t="n">
+    <row r="7">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Render Manual Deploy Mode</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>Prevents surprise container reboots while an active trade is running.</t>
         </is>
       </c>
-      <c r="D7" s="26" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Render will never restart mid-trade on git push. Manual deploy only when flat.</t>
         </is>
       </c>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Infrastructure Stability</t>
         </is>
       </c>
-      <c r="F7" s="27" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Configured &amp; Active</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="24" t="n">
+    <row r="8">
+      <c r="A8" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="25" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Startup Position Reconciler</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Prevents lost positions if an unexpected reboot ever occurs.</t>
         </is>
       </c>
-      <c r="D8" s="26" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>On boot, queries Delta API for open positions and auto-adopts them with brackets.</t>
         </is>
       </c>
-      <c r="E8" s="27" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Crash Recovery Shield</t>
         </is>
       </c>
-      <c r="F8" s="27" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Verified &amp; Deployed</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="44" customHeight="1">
-      <c r="A9" s="24" t="n">
+    <row r="9">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Micro-Wick Cushion on SL</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Prevents market maker liquidity sweeps from hunting tight stops.</t>
         </is>
       </c>
-      <c r="D9" s="26" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Adds 0.08% / 0.20 ATR buffer beyond Higher Highs / Lower Lows.</t>
         </is>
       </c>
-      <c r="E9" s="27" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Stop-Out Reduction</t>
         </is>
       </c>
-      <c r="F9" s="27" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Verified &amp; Tested (6/6 Tests)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="44" customHeight="1">
-      <c r="A10" s="24" t="n">
+    <row r="10">
+      <c r="A10" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="25" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Pre-Flight Spread Guard</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Prevents bad fills and slippage during thin order book liquidity.</t>
         </is>
       </c>
-      <c r="D10" s="26" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Checks live spread; pauses 3s if spread exceeds 12 bps (0.12%).</t>
         </is>
       </c>
-      <c r="E10" s="27" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Slippage Protection</t>
         </is>
       </c>
-      <c r="F10" s="27" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Verified &amp; Tested</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="44" customHeight="1">
-      <c r="A11" s="24" t="n">
+    <row r="11">
+      <c r="A11" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>11:59 PM IST Midnight Rollover</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Prevents loss rollover confusion across daily trading sessions.</t>
         </is>
       </c>
-      <c r="D11" s="26" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>Resets daily loss to ₹0.00 at 23:59 IST, restoring the full ₹201 budget automatically.</t>
         </is>
       </c>
-      <c r="E11" s="27" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Session Discipline</t>
         </is>
       </c>
-      <c r="F11" s="27" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Verified &amp; Tested</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="A12" s="24" t="n">
+    <row r="12">
+      <c r="A12" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="25" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Dynamic Margin Band (₹3,000 – ₹4,500)</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Prevents Delta Exchange 'insufficient_margin' 400 rejections when equity drops.</t>
         </is>
       </c>
-      <c r="D12" s="26" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>Auto-syncs with live Delta wallet balance and uses 95% collateral cushion. Allows all trades between ₹3,000 and ₹4,500.</t>
         </is>
       </c>
-      <c r="E12" s="27" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Margin Rejection Shield</t>
         </is>
       </c>
-      <c r="F12" s="27" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Verified &amp; Tested (5/5 Tests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Limit Order TP Execution (0.02% Maker)</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>Prevents high taker fee erosion on profitable take profit exits.</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Routes TP orders as Post-Only Limit orders, saving 60% in exchange fees.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Fee Retention Shield</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Verified &amp; Live (Commit c33c614)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record XRP and AVAX live trades in journal with chart proof and disabled bot post-mortem
</commit_message>
<xml_diff>
--- a/Real_Money_Trades.xlsx
+++ b/Real_Money_Trades.xlsx
@@ -585,8 +585,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:N10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
@@ -618,7 +618,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -652,9 +651,14 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3 Live Trades</t>
+        </is>
+      </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1 Live Trade</t>
+          <t>-₹103.69 Net (-₹139.68 Today)</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -662,9 +666,14 @@
           <t>+₹35.99 Net</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PnL: -₹230.80 | Fees: ₹81.74</t>
+        </is>
+      </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>₹201.00 Max</t>
+          <t>Autonomous Bot OFF (Manual Control)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -683,7 +692,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
@@ -813,6 +821,126 @@
       <c r="N8" s="9" t="inlineStr">
         <is>
           <t>1st Live Win! Model 10 Sniper Long triggered in 31.9% discount zone after $2,465.05 SSL sweep &amp; 83.4% body displacement. Rocketed to $2,486.10 (+1.61R peak). 50% partial TP executed @ $2,478.00 (+₹41.99 gross), remaining 5.38 contracts exited on trailing stop @ $2,468.15 (+₹16.00). Net +₹35.99 credited (+₹30.00 after ₹22 fees).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09-09-2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>XRPUSD</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MODEL_10 (Institutional Sniper)</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1.4517</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.4401</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1.4725</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.4807</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1.4401 (SL)</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>LOSS (Stop Loss Hit)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>-1.00R</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>-93.68000000000001</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>XRP Long took stop loss on market pull back. Loss -₹93.68.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09-09-2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>AVAXUSD</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>MODEL_8 (Liquidity Sweep Reversal)</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>7.9264</v>
+      </c>
+      <c r="G10" t="n">
+        <v>7.888</v>
+      </c>
+      <c r="H10" t="n">
+        <v>7.9918</v>
+      </c>
+      <c r="I10" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>7.9100 (Bot Premature Close)</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>PREMATURE BOT EXIT (Strangled on 5M Wick)</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>-0.48R</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>-46</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>AVAX Long 29 contracts filled @ .9264. Surged to .946 (+0.57R profit). Spidy trailing stop engine ratcheted internally to .91 on 5M swing and market-closed on quick wick to .898, while user manual SL at .888 was NEVER touched! Immediately rebounded with massive lower wick. Bot execution permanently disabled.</t>
         </is>
       </c>
     </row>
@@ -832,7 +960,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -857,7 +985,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -1051,7 +1178,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
@@ -1068,7 +1195,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: finalize Real_Money_Trades.xlsx row formatting
</commit_message>
<xml_diff>
--- a/Real_Money_Trades.xlsx
+++ b/Real_Money_Trades.xlsx
@@ -661,9 +661,14 @@
           <t>-₹103.69 Net (-₹139.68 Today)</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>₹201.00 Max</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>+₹35.99 Net</t>
+          <t>₹201.00 (Restored)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -676,21 +681,9 @@
           <t>Autonomous Bot OFF (Manual Control)</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>₹201.00 (Full Restored)</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>₹4,610.84 INR</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Armed &amp; 100% Operational</t>
-        </is>
-      </c>
+      <c r="H5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: sync Real_Money_Trades.xlsx with Delta Exchange India live figures
</commit_message>
<xml_diff>
--- a/Real_Money_Trades.xlsx
+++ b/Real_Money_Trades.xlsx
@@ -18,11 +18,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="₹#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.0000"/>
+    <numFmt numFmtId="167" formatCode="₹#,##0.00;[Red]-₹#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,8 +90,26 @@
       <color rgb="001E293B"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00475569"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +144,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAFC"/>
         <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
+        <bgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -167,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -218,6 +244,36 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -631,17 +687,17 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>DAILY LOSS BUDGET</t>
+          <t>TODAY'S PnL (09-09)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>REMAINING RISK QUOTA</t>
+          <t>FEES PAID (DELTA)</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>LIVE EQUITY (+₹300 DEPOSIT)</t>
+          <t>TOTAL DRAWDOWN</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -651,39 +707,36 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>3 Live Trades</t>
-        </is>
-      </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>-₹103.69 Net (-₹139.68 Today)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>₹201.00 Max</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>₹201.00 (Restored)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>PnL: -₹230.80 | Fees: ₹81.74</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Autonomous Bot OFF (Manual Control)</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
+          <t>5 Closed Trades</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>-₹230.80</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>-₹139.68</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>₹81.74</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>-₹312.54</t>
+        </is>
+      </c>
+      <c r="L5" s="21" t="inlineStr">
+        <is>
+          <t>Autonomous Bot OFF</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -817,123 +870,123 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="n">
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>09-09-2026</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>XRPUSD</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr">
         <is>
           <t>LONG</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>MODEL_10 (Institutional Sniper)</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="25" t="n">
         <v>1.4517</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="25" t="n">
         <v>1.4401</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="25" t="n">
         <v>1.4725</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="25" t="n">
         <v>1.4807</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>1.4401 (SL)</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
+        <is>
+          <t>1.4401 (Stop Loss Hit)</t>
+        </is>
+      </c>
+      <c r="K9" s="23" t="inlineStr">
         <is>
           <t>LOSS (Stop Loss Hit)</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" s="22" t="inlineStr">
         <is>
           <t>-1.00R</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="26" t="n">
         <v>-93.68000000000001</v>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>XRP Long took stop loss on market pull back. Loss -₹93.68.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
+      <c r="N9" s="27" t="inlineStr">
+        <is>
+          <t>XRPUSD Long entered @ $1.4517. Morning market-wide pullback dropped price to $1.4401 where disciplined Stop Loss cleanly executed. Risk strictly managed at 1.00R (-₹93.68).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>09-09-2026</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>AVAXUSD</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>LONG</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>MODEL_8 (Liquidity Sweep Reversal)</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="25" t="n">
         <v>7.9264</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="25" t="n">
         <v>7.888</v>
       </c>
-      <c r="H10" t="n">
-        <v>7.9918</v>
-      </c>
-      <c r="I10" t="n">
+      <c r="H10" s="25" t="n">
+        <v>7.958</v>
+      </c>
+      <c r="I10" s="25" t="n">
         <v>8.039999999999999</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>7.9100 (Bot Premature Close)</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
+        <is>
+          <t>7.9100 (Autonomous Bot Premature Exit)</t>
+        </is>
+      </c>
+      <c r="K10" s="23" t="inlineStr">
         <is>
           <t>PREMATURE BOT EXIT (Strangled on 5M Wick)</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>-0.48R</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
+      <c r="L10" s="22" t="inlineStr">
+        <is>
+          <t>-0.48R (Peak: +0.70R @ $7.9528)</t>
+        </is>
+      </c>
+      <c r="M10" s="26" t="n">
         <v>-46</v>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>AVAX Long 29 contracts filled @ .9264. Surged to .946 (+0.57R profit). Spidy trailing stop engine ratcheted internally to .91 on 5M swing and market-closed on quick wick to .898, while user manual SL at .888 was NEVER touched! Immediately rebounded with massive lower wick. Bot execution permanently disabled.</t>
+      <c r="N10" s="27" t="inlineStr">
+        <is>
+          <t>AVAX Long 29 contracts filled @ $7.9264. Surged to $7.9460 (+0.57R profit). Spidy trailing engine ratcheted internally to $7.9100 on 5M swing and market-closed on quick wick to $7.8980, while user manual SL at $7.8880 was NEVER touched! Immediately after bot closed trade, price formed massive lower wick and exploded straight to $7.9528 target line! Bot execution permanently disabled. Breathing room guard (&lt; 0.8R) deployed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(execution): re-arm live autonomous execution on Delta Exchange with all institutional safeguards active
</commit_message>
<xml_diff>
--- a/Real_Money_Trades.xlsx
+++ b/Real_Money_Trades.xlsx
@@ -732,9 +732,9 @@
           <t>-₹312.54</t>
         </is>
       </c>
-      <c r="L5" s="21" t="inlineStr">
-        <is>
-          <t>Autonomous Bot OFF</t>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Armed &amp; 100% Operational</t>
         </is>
       </c>
     </row>

</xml_diff>